<commit_message>
fix: browser robustness for CUHK/CityU/Caritas + correct UNHCR URL
From the Jul 24 Actions run log, four blocked sites failed for fixable
reasons rather than real anti-bot walls:

- CUHK / CityU: 'Execution context was destroyed' — page.evaluate raced
  a JS navigation. Added safeEvaluate() with wait-and-retry, used for
  every extraction
- Caritas: goto timed out at 45s — retry once at 75s
- JS-app pages returning <200 chars on first extraction now get a 6s
  second chance (HKMU e-tender shell)
- UNHCR: etenderbox.unhcr.org no longer resolves — organisations.csv now
  points at the global invitations-to-bid page; xlsx regenerated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPZ7VGAy3s2eRme386vk
</commit_message>
<xml_diff>
--- a/data/Tender_Organisations.xlsx
+++ b/data/Tender_Organisations.xlsx
@@ -4476,7 +4476,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>https://etenderbox.unhcr.org/</t>
+          <t>https://www.unhcr.org/invitations-bid.html</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -4486,17 +4486,17 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>待驗證</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-07] 修正URL:舊 etenderbox.unhcr.org 域名已無法解析</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>⭐⭐⭐ 高相關|UNHCR香港辦事處負責私營部門夥伴(籌款)業務,定期為香港市場公開招標。WebFetch被擋(代理DNS/403),但搜尋結果證實eTenderBox為UNHCR官方公開投標平台,且曾刊登「Establishment of a Frame Agreement for the Provision of Digital Marketing Services for UNHCR Private Sector Partnerships in Hong Kong SAR」數碼營銷框架協議招標。屬全球平台,監察時需篩選Hong Kong;對數碼營銷及F2F籌款代理高度相關。</t>
+          <t>⭐⭐⭐ 高相關|UNHCR香港辦事處負責私營部門夥伴(籌款)業務,定期為香港市場公開招標。WebFetch被擋(代理DNS/403),但搜尋結果證實eTenderBox為UNHCR官方公開投標平台,且曾刊登「Establishment of a Frame Agreement for the Provision of Digital Marketing Services for UNHCR Private Sector Partnerships in Hong Kong SAR」數碼營銷框架協議招標。屬全球平台,監察時需篩選Hong Kong;對數碼營銷及F2F籌款代理高度相關。 | 2026-08-07 更新為 UNHCR 全球 bidding 頁</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: 2026-08-23 URL 健康檢查 — 17 個狀態更新
14 個機構由受阻轉為正常(房委會、海洋公園、香港郵政、生產力局、
城大、手球總會等);HKEX 及新生精神康復會招標頁 404 待修;
保險業監管局及 UNHCR 確認 403 受阻。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPZ7VGAy3s2eRme386vk
</commit_message>
<xml_diff>
--- a/data/Tender_Organisations.xlsx
+++ b/data/Tender_Organisations.xlsx
@@ -802,12 +802,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:30] 🌐 網絡連線超時，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -998,12 +998,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>受阻</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:31] 掃描完成：暫無符合條件之新標書</t>
+          <t>[2026-08-23] 狀態更新:受阻(HTTP 403)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1026,12 +1026,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:31] 🔒 網站防爬蟲攔截 (403)，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1418,12 +1418,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:32] 🌐 網絡連線超時，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:32] 🌐 網絡連線超時，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:33] 🔒 網站防爬蟲攔截 (403)，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3602,12 +3602,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>[2026-07-09 12:38] 🌐 網絡連線超時，已加入綜合報告提示手動檢查</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -3974,12 +3974,12 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -4134,12 +4134,12 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -4262,12 +4262,12 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>失效</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:失效(HTTP 404)</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -4454,12 +4454,12 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -4486,12 +4486,12 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>待驗證</t>
+          <t>受阻</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>[2026-08-07] 修正URL:舊 etenderbox.unhcr.org 域名已無法解析</t>
+          <t>[2026-08-23] 狀態更新:受阻(HTTP 403)</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -5062,12 +5062,12 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -5350,12 +5350,12 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -5446,12 +5446,12 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>失效</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:失效(HTTP 404)</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -5510,12 +5510,12 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
@@ -5766,12 +5766,12 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 狀態更新:正常(HTTP 200)</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: 依 2026-08-23 Playwright 實戰結果修正狀態
- HKEX、新生精神康復會由「失效」更正為「受阻」(curl 404 但真瀏覽器
  抓到,補漏掃描已覆蓋)
- UNHCR 再換 URL:invitations-bid.html 對 bot 無限 redirect
- 明愛確認 URL 無誤,純粹伺服器極慢

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPZ7VGAy3s2eRme386vk
</commit_message>
<xml_diff>
--- a/data/Tender_Organisations.xlsx
+++ b/data/Tender_Organisations.xlsx
@@ -4262,12 +4262,12 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>失效</t>
+          <t>受阻</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>[2026-08-23] 狀態更新:失效(HTTP 404)</t>
+          <t>[2026-08-23] 更正:curl 404 但真瀏覽器抓到,Playwright 補漏掃描已覆蓋</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>https://www.unhcr.org/invitations-bid.html</t>
+          <t>https://www.unhcr.org/get-involved/work-us/become-supplier</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -4486,12 +4486,12 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>受阻</t>
+          <t>待驗證</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>[2026-08-23] 狀態更新:受阻(HTTP 403)</t>
+          <t>[2026-08-23] 再修正URL:invitations-bid.html 對 bot 無限redirect,改用 become-supplier 頁</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -5446,12 +5446,12 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>失效</t>
+          <t>受阻</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>[2026-08-23] 狀態更新:失效(HTTP 404)</t>
+          <t>[2026-08-23] 更正:curl 404 但真瀏覽器抓到,Playwright 補漏掃描已覆蓋</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>[2026-07-14] 新增機構,待首次掃描</t>
+          <t>[2026-08-23] 伺服器極慢(75秒都load唔到),URL經搜尋確認無誤,標受阻待間歇性重試</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: force-browser flag for JS-rendered sites; add OpenTender.hk aggregator
OpenTender.hk indexes all HK government and public-body open tenders
daily but renders client-side — its large HTML shell passed plainFetch
so it never reached the browser path. Organisations whose 備註 contains
強制瀏覽器 now go straight to Playwright. Added the aggregator as a
184th watch target: a safety net for tenders from bodies outside the
curated list.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPZ7VGAy3s2eRme386vk
</commit_message>
<xml_diff>
--- a/data/Tender_Organisations.xlsx
+++ b/data/Tender_Organisations.xlsx
@@ -10,7 +10,7 @@
     <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'list'!$A$1:$F$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'list'!$A$1:$F$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5876,8 +5876,40 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>OpenTender.hk 全港招標聚合索引</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>https://opentender.hk/status/active</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>聚合索引</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>待驗證</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>[2026-08-31] 新增:每日更新嘅全港政府+公營機構公開招標索引,作為183名單以外嘅保險網</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>⭐ 高價值聚合源|JS渲染站,強制瀏覽器掃描。捕捉唔喺監察名單嘅機構出嘅 marketing/PR 類標書。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F184"/>
+  <autoFilter ref="A1:F185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>